<commit_message>
Update data for coverage and introduction
</commit_message>
<xml_diff>
--- a/data/HPV_introduction.xlsx
+++ b/data/HPV_introduction.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22125" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23292" uniqueCount="442">
   <si>
     <t xml:space="preserve">ISO_3_CODE</t>
   </si>
@@ -52,7 +52,7 @@
     <t xml:space="preserve">HPV</t>
   </si>
   <si>
-    <t xml:space="preserve">HPV (Human Papilloma Virus) vaccine</t>
+    <t xml:space="preserve">HPV (Human papillomavirus) vaccine</t>
   </si>
   <si>
     <t xml:space="preserve">No</t>
@@ -787,7 +787,7 @@
     <t xml:space="preserve">NRU</t>
   </si>
   <si>
-    <t xml:space="preserve">Nauru</t>
+    <t xml:space="preserve">Naoero</t>
   </si>
   <si>
     <t xml:space="preserve">NPL</t>
@@ -1240,19 +1240,19 @@
     <t xml:space="preserve">Yes (D)</t>
   </si>
   <si>
-    <t xml:space="preserve">Exported: 2025-10-10 11:37 UTC</t>
+    <t xml:space="preserve">Exported: 2026-30-7 8:8 UTC</t>
   </si>
   <si>
     <t xml:space="preserve">Definition</t>
   </si>
   <si>
-    <t xml:space="preserve">Data presented shows introduction status of the selected vaccine over time.</t>
+    <t xml:space="preserve">Data presented shows introduction status of HPV (human papillomavirus) vaccine over time.</t>
   </si>
   <si>
     <t xml:space="preserve">Data collection information</t>
   </si>
   <si>
-    <t xml:space="preserve">The data shows the number of countries having introduced or that will introduce per year and for selected vaccine(s). The data is requested annually through the WHO/UNICEF Joint Reporting Form on Immunization (JRF), and is queried quarterly through WHO Regional Offices to be updated regularly.</t>
+    <t xml:space="preserve">The data shows the number of countries having introduced HPV (human papillomavirus) vaccine per year. The data is requested annually through the WHO/UNICEF Joint Reporting Form on Immunization (JRF).</t>
   </si>
   <si>
     <t xml:space="preserve">Rationale</t>
@@ -1276,10 +1276,10 @@
     <t xml:space="preserve">Advanced filter</t>
   </si>
   <si>
-    <t xml:space="preserve">DEVELOPMENT STATUS: World Economic Situation and Prospects 2025
-GAVI: Eligibility status
+    <t xml:space="preserve">Development Status: World Economic Situation and Prospects 2026
+Gavi (according to Gavi 5.0 strategic framework): Eligibility status
 UNICEF: Regional offices
-WORLD BANK INCOME STATUS: Country classification by income</t>
+World Bank income status: Country classification by income</t>
   </si>
   <si>
     <t xml:space="preserve">Data type</t>
@@ -1295,7 +1295,7 @@
 Yes (P): Vaccine is administered only in certain regions of the country
 Yes (R): Vaccine is not administered to the entire population, only to specific risk groups
 Yes (A): Vaccine is administered to adolescents
-Yes (O): Vaccine is administered to in case of outbreaks
+Yes (O): Vaccine is administered in case of outbreaks
 High risk: Vaccine is administered in high risk areas
 No: Vaccine is not administered
 No (D): Vaccine is not in the schedule but demonstration projects are ongoing
@@ -1306,7 +1306,11 @@
     <t xml:space="preserve">Method of estimation</t>
   </si>
   <si>
-    <t xml:space="preserve">WHO displays data as reported by national authorities.</t>
+    <t xml:space="preserve">WHO displays data as reported by national authorities.
+Pending data (e.g., current reporting year):
+- If a country’s most recent official report indicates that a vaccine was introduced (Yes), the value is carried forward from the last available reported year until official data for that year are received.
+- If a country’s most recent official report indicates that a vaccine was not introduced (No), the value for the pending year is displayed as ND (No data available) until official data are received.
+- Once official data are received, reported values replace carried forward or ND values.</t>
   </si>
   <si>
     <t xml:space="preserve">Preferred data source</t>
@@ -1318,13 +1322,20 @@
     <t xml:space="preserve">Data collection source</t>
   </si>
   <si>
-    <t xml:space="preserve">WHO/UNICEF Joint Reporting Form on Immunization (JRF), WHO Regional and Country offices</t>
+    <t xml:space="preserve">WHO/UNICEF Joint Reporting Form on Immunization (JRF), officially reported data to WHO/UNICEF
+Data from other official sources, including information formally reported by national authorities to WHO, PAHO, UNICEF, or partners, and data published on official government websites, may be included following technical review and validation.</t>
   </si>
   <si>
-    <t xml:space="preserve">Data frequency</t>
+    <t xml:space="preserve">Expected frequency of data collection</t>
   </si>
   <si>
-    <t xml:space="preserve">Quarterly</t>
+    <t xml:space="preserve">Data are collected annually through the WHO/UNICEF Joint Reporting Form on Immunization (JRF) exercise (occurring in Q1-Q2 of each year).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expected frequency of data dissemination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data (including historical data) are updated and made available as received.</t>
   </si>
   <si>
     <t xml:space="preserve">Data collected from</t>
@@ -1337,16 +1348,19 @@
     <t xml:space="preserve">Limitations</t>
   </si>
   <si>
-    <t xml:space="preserve">Although countries report having introduced select vaccines in national immunization schedules, it does not mean children are vaccinated.</t>
+    <t xml:space="preserve">Although countries report having introduced select vaccines in national immunization schedules, this does not mean children are vaccinated.</t>
   </si>
   <si>
     <t xml:space="preserve">Comments</t>
   </si>
   <si>
-    <t xml:space="preserve">Please inform WHO Global Monitoring team of incorrect or missing information at: vpdata@who.int.</t>
+    <t xml:space="preserve">Please inform the WHO Global Monitoring &amp; Surveillance Team of incorrect or missing information at: vpdata@who.int.</t>
   </si>
   <si>
     <t xml:space="preserve">https://app.powerbi.com/view?r=eyJrIjoiNDIxZTFkZGUtMDQ1Ny00MDZkLThiZDktYWFlYTdkOGU2NDcwIiwidCI6ImY2MTBjMGI3LWJkMjQtNGIzOS04MTBiLTNkYzI4MGFmYjU5MCIsImMiOjh9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/docs/librariesprovider21/additional-datasets/vaccine-introduction-official.pptx?sfvrsn=3e65a61c_1</t>
   </si>
 </sst>
 </file>
@@ -1410,10 +1424,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3683"/>
+  <dimension ref="A1:G3877"/>
   <sheetFormatPr x14ac:dyDescent="0.25" customHeight="1" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="30.714285714285715" bestFit="1"/>
+    <col min="1" max="1" customWidth="1" width="27.714285714285715" bestFit="1"/>
     <col min="2" max="2" customWidth="1" width="52.714285714285715" bestFit="1"/>
   </cols>
   <sheetData>
@@ -3265,7 +3279,7 @@
         <v>176</v>
       </c>
       <c r="C81" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D81" t="n">
         <v>2006</v>
@@ -7704,7 +7718,7 @@
         <v>176</v>
       </c>
       <c r="C274" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D274" t="n">
         <v>2007</v>
@@ -12143,7 +12157,7 @@
         <v>176</v>
       </c>
       <c r="C467" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D467" t="n">
         <v>2008</v>
@@ -16582,7 +16596,7 @@
         <v>176</v>
       </c>
       <c r="C660" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D660" t="n">
         <v>2009</v>
@@ -21021,7 +21035,7 @@
         <v>176</v>
       </c>
       <c r="C853" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D853" t="n">
         <v>2010</v>
@@ -25460,7 +25474,7 @@
         <v>176</v>
       </c>
       <c r="C1046" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D1046" t="n">
         <v>2011</v>
@@ -29922,7 +29936,7 @@
         <v>176</v>
       </c>
       <c r="C1240" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D1240" t="n">
         <v>2012</v>
@@ -34384,7 +34398,7 @@
         <v>176</v>
       </c>
       <c r="C1434" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D1434" t="n">
         <v>2013</v>
@@ -38846,7 +38860,7 @@
         <v>176</v>
       </c>
       <c r="C1628" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D1628" t="n">
         <v>2014</v>
@@ -43308,7 +43322,7 @@
         <v>176</v>
       </c>
       <c r="C1822" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D1822" t="n">
         <v>2015</v>
@@ -47770,7 +47784,7 @@
         <v>176</v>
       </c>
       <c r="C2016" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D2016" t="n">
         <v>2016</v>
@@ -52232,7 +52246,7 @@
         <v>176</v>
       </c>
       <c r="C2210" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D2210" t="n">
         <v>2017</v>
@@ -56694,7 +56708,7 @@
         <v>176</v>
       </c>
       <c r="C2404" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D2404" t="n">
         <v>2018</v>
@@ -61156,7 +61170,7 @@
         <v>176</v>
       </c>
       <c r="C2598" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D2598" t="n">
         <v>2019</v>
@@ -65618,7 +65632,7 @@
         <v>176</v>
       </c>
       <c r="C2792" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D2792" t="n">
         <v>2020</v>
@@ -70080,7 +70094,7 @@
         <v>176</v>
       </c>
       <c r="C2986" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D2986" t="n">
         <v>2021</v>
@@ -74542,7 +74556,7 @@
         <v>176</v>
       </c>
       <c r="C3180" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D3180" t="n">
         <v>2022</v>
@@ -79004,7 +79018,7 @@
         <v>176</v>
       </c>
       <c r="C3374" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D3374" t="n">
         <v>2023</v>
@@ -83466,7 +83480,7 @@
         <v>176</v>
       </c>
       <c r="C3568" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D3568" t="n">
         <v>2024</v>
@@ -84536,7 +84550,7 @@
         <v>11</v>
       </c>
       <c r="G3614" t="s">
-        <v>403</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3615" x14ac:dyDescent="0.25">
@@ -86105,6 +86119,4468 @@
     </row>
     <row r="3683" x14ac:dyDescent="0.25">
       <c r="A3683" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3683" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3683" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3683" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3683" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3683" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3683" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3684" x14ac:dyDescent="0.25">
+      <c r="A3684" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3684" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3684" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3684" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3684" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3684" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3684" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3685" x14ac:dyDescent="0.25">
+      <c r="A3685" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3685" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3685" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3685" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3685" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3685" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3685" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3686" x14ac:dyDescent="0.25">
+      <c r="A3686" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3686" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3686" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3686" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3686" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3686" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3686" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3687" x14ac:dyDescent="0.25">
+      <c r="A3687" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3687" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3687" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3687" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3687" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3687" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3687" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3688" x14ac:dyDescent="0.25">
+      <c r="A3688" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3688" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3688" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3688" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3688" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3688" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3688" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3689" x14ac:dyDescent="0.25">
+      <c r="A3689" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3689" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3689" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3689" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3689" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3689" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3689" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3690" x14ac:dyDescent="0.25">
+      <c r="A3690" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3690" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3690" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3690" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3690" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3690" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3690" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3691" x14ac:dyDescent="0.25">
+      <c r="A3691" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3691" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3691" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3691" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3691" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3691" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3691" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3692" x14ac:dyDescent="0.25">
+      <c r="A3692" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3692" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3692" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3692" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3692" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3692" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3692" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3693" x14ac:dyDescent="0.25">
+      <c r="A3693" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3693" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3693" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3693" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3693" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3693" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3693" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3694" x14ac:dyDescent="0.25">
+      <c r="A3694" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3694" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3694" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3694" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3694" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3694" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3694" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3695" x14ac:dyDescent="0.25">
+      <c r="A3695" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3695" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3695" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3695" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3695" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3695" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3695" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3696" x14ac:dyDescent="0.25">
+      <c r="A3696" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3696" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3696" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3696" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3696" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3696" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3696" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3697" x14ac:dyDescent="0.25">
+      <c r="A3697" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3697" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3697" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3697" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3697" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3697" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3697" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3698" x14ac:dyDescent="0.25">
+      <c r="A3698" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3698" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3698" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3698" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3698" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3698" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3698" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3699" x14ac:dyDescent="0.25">
+      <c r="A3699" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3699" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3699" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3699" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3699" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3699" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3699" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3700" x14ac:dyDescent="0.25">
+      <c r="A3700" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3700" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3700" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3700" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3700" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3700" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3700" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3701" x14ac:dyDescent="0.25">
+      <c r="A3701" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3701" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3701" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3701" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3701" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3701" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3701" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3702" x14ac:dyDescent="0.25">
+      <c r="A3702" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3702" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3702" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3702" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3702" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3702" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3702" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3703" x14ac:dyDescent="0.25">
+      <c r="A3703" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3703" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3703" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3703" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3703" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3703" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3703" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3704" x14ac:dyDescent="0.25">
+      <c r="A3704" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3704" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3704" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3704" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3704" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3704" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3704" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3705" x14ac:dyDescent="0.25">
+      <c r="A3705" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3705" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3705" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3705" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3705" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3705" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3705" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3706" x14ac:dyDescent="0.25">
+      <c r="A3706" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3706" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3706" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3706" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3706" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3706" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3706" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3707" x14ac:dyDescent="0.25">
+      <c r="A3707" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3707" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3707" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3707" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3707" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3707" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3707" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3708" x14ac:dyDescent="0.25">
+      <c r="A3708" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3708" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3708" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3708" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3708" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3708" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3708" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3709" x14ac:dyDescent="0.25">
+      <c r="A3709" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3709" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3709" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3709" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3709" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3709" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3709" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3710" x14ac:dyDescent="0.25">
+      <c r="A3710" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3710" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3710" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3710" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3710" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3710" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3710" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3711" x14ac:dyDescent="0.25">
+      <c r="A3711" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3711" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3711" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3711" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3711" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3711" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3711" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3712" x14ac:dyDescent="0.25">
+      <c r="A3712" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3712" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3712" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3712" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3712" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3712" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3712" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3713" x14ac:dyDescent="0.25">
+      <c r="A3713" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3713" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3713" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3713" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3713" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3713" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3713" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3714" x14ac:dyDescent="0.25">
+      <c r="A3714" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3714" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3714" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3714" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3714" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3714" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3714" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3715" x14ac:dyDescent="0.25">
+      <c r="A3715" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3715" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3715" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3715" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3715" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3715" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3715" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3716" x14ac:dyDescent="0.25">
+      <c r="A3716" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3716" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3716" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3716" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3716" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3716" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3716" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3717" x14ac:dyDescent="0.25">
+      <c r="A3717" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3717" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3717" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3717" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3717" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3717" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3717" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3718" x14ac:dyDescent="0.25">
+      <c r="A3718" t="s">
+        <v>86</v>
+      </c>
+      <c r="B3718" t="s">
+        <v>87</v>
+      </c>
+      <c r="C3718" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3718" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3718" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3718" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3718" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3719" x14ac:dyDescent="0.25">
+      <c r="A3719" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3719" t="s">
+        <v>89</v>
+      </c>
+      <c r="C3719" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3719" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3719" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3719" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3719" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3720" x14ac:dyDescent="0.25">
+      <c r="A3720" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3720" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3720" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3720" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3720" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3720" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3720" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3721" x14ac:dyDescent="0.25">
+      <c r="A3721" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3721" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3721" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3721" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3721" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3721" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3721" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3722" x14ac:dyDescent="0.25">
+      <c r="A3722" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3722" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3722" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3722" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3722" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3722" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3722" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3723" x14ac:dyDescent="0.25">
+      <c r="A3723" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3723" t="s">
+        <v>97</v>
+      </c>
+      <c r="C3723" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3723" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3723" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3723" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3723" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3724" x14ac:dyDescent="0.25">
+      <c r="A3724" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3724" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3724" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3724" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3724" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3724" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3724" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3725" x14ac:dyDescent="0.25">
+      <c r="A3725" t="s">
+        <v>100</v>
+      </c>
+      <c r="B3725" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3725" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3725" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3725" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3725" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3725" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3726" x14ac:dyDescent="0.25">
+      <c r="A3726" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3726" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3726" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3726" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3726" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3726" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3726" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3727" x14ac:dyDescent="0.25">
+      <c r="A3727" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3727" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3727" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3727" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3727" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3727" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3727" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3728" x14ac:dyDescent="0.25">
+      <c r="A3728" t="s">
+        <v>106</v>
+      </c>
+      <c r="B3728" t="s">
+        <v>107</v>
+      </c>
+      <c r="C3728" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3728" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3728" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3728" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3728" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3729" x14ac:dyDescent="0.25">
+      <c r="A3729" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3729" t="s">
+        <v>109</v>
+      </c>
+      <c r="C3729" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3729" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3729" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3729" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3729" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3730" x14ac:dyDescent="0.25">
+      <c r="A3730" t="s">
+        <v>110</v>
+      </c>
+      <c r="B3730" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3730" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3730" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3730" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3730" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3730" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3731" x14ac:dyDescent="0.25">
+      <c r="A3731" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3731" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3731" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3731" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3731" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3731" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3731" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3732" x14ac:dyDescent="0.25">
+      <c r="A3732" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3732" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3732" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3732" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3732" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3732" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3732" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3733" x14ac:dyDescent="0.25">
+      <c r="A3733" t="s">
+        <v>116</v>
+      </c>
+      <c r="B3733" t="s">
+        <v>117</v>
+      </c>
+      <c r="C3733" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3733" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3733" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3733" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3733" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3734" x14ac:dyDescent="0.25">
+      <c r="A3734" t="s">
+        <v>118</v>
+      </c>
+      <c r="B3734" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3734" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3734" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3734" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3734" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3734" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3735" x14ac:dyDescent="0.25">
+      <c r="A3735" t="s">
+        <v>120</v>
+      </c>
+      <c r="B3735" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3735" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3735" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3735" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3735" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3735" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3736" x14ac:dyDescent="0.25">
+      <c r="A3736" t="s">
+        <v>122</v>
+      </c>
+      <c r="B3736" t="s">
+        <v>123</v>
+      </c>
+      <c r="C3736" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3736" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3736" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3736" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3736" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3737" x14ac:dyDescent="0.25">
+      <c r="A3737" t="s">
+        <v>124</v>
+      </c>
+      <c r="B3737" t="s">
+        <v>125</v>
+      </c>
+      <c r="C3737" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3737" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3737" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3737" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3737" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3738" x14ac:dyDescent="0.25">
+      <c r="A3738" t="s">
+        <v>126</v>
+      </c>
+      <c r="B3738" t="s">
+        <v>127</v>
+      </c>
+      <c r="C3738" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3738" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3738" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3738" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3738" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3739" x14ac:dyDescent="0.25">
+      <c r="A3739" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3739" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3739" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3739" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3739" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3739" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3739" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3740" x14ac:dyDescent="0.25">
+      <c r="A3740" t="s">
+        <v>130</v>
+      </c>
+      <c r="B3740" t="s">
+        <v>131</v>
+      </c>
+      <c r="C3740" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3740" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3740" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3740" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3740" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3741" x14ac:dyDescent="0.25">
+      <c r="A3741" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3741" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3741" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3741" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3741" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3741" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3741" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3742" x14ac:dyDescent="0.25">
+      <c r="A3742" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3742" t="s">
+        <v>135</v>
+      </c>
+      <c r="C3742" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3742" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3742" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3742" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3742" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3743" x14ac:dyDescent="0.25">
+      <c r="A3743" t="s">
+        <v>136</v>
+      </c>
+      <c r="B3743" t="s">
+        <v>137</v>
+      </c>
+      <c r="C3743" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3743" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3743" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3743" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3743" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3744" x14ac:dyDescent="0.25">
+      <c r="A3744" t="s">
+        <v>138</v>
+      </c>
+      <c r="B3744" t="s">
+        <v>139</v>
+      </c>
+      <c r="C3744" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3744" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3744" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3744" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3744" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3745" x14ac:dyDescent="0.25">
+      <c r="A3745" t="s">
+        <v>140</v>
+      </c>
+      <c r="B3745" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3745" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3745" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3745" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3745" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3745" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3746" x14ac:dyDescent="0.25">
+      <c r="A3746" t="s">
+        <v>143</v>
+      </c>
+      <c r="B3746" t="s">
+        <v>144</v>
+      </c>
+      <c r="C3746" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3746" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3746" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3746" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3746" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3747" x14ac:dyDescent="0.25">
+      <c r="A3747" t="s">
+        <v>145</v>
+      </c>
+      <c r="B3747" t="s">
+        <v>146</v>
+      </c>
+      <c r="C3747" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3747" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3747" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3747" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3747" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3748" x14ac:dyDescent="0.25">
+      <c r="A3748" t="s">
+        <v>147</v>
+      </c>
+      <c r="B3748" t="s">
+        <v>148</v>
+      </c>
+      <c r="C3748" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3748" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3748" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3748" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3748" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3749" x14ac:dyDescent="0.25">
+      <c r="A3749" t="s">
+        <v>149</v>
+      </c>
+      <c r="B3749" t="s">
+        <v>150</v>
+      </c>
+      <c r="C3749" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3749" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3749" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3749" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3749" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3750" x14ac:dyDescent="0.25">
+      <c r="A3750" t="s">
+        <v>151</v>
+      </c>
+      <c r="B3750" t="s">
+        <v>152</v>
+      </c>
+      <c r="C3750" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3750" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3750" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3750" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3750" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3751" x14ac:dyDescent="0.25">
+      <c r="A3751" t="s">
+        <v>153</v>
+      </c>
+      <c r="B3751" t="s">
+        <v>154</v>
+      </c>
+      <c r="C3751" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3751" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3751" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3751" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3751" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3752" x14ac:dyDescent="0.25">
+      <c r="A3752" t="s">
+        <v>155</v>
+      </c>
+      <c r="B3752" t="s">
+        <v>156</v>
+      </c>
+      <c r="C3752" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3752" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3752" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3752" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3752" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3753" x14ac:dyDescent="0.25">
+      <c r="A3753" t="s">
+        <v>157</v>
+      </c>
+      <c r="B3753" t="s">
+        <v>158</v>
+      </c>
+      <c r="C3753" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3753" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3753" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3753" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3753" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3754" x14ac:dyDescent="0.25">
+      <c r="A3754" t="s">
+        <v>159</v>
+      </c>
+      <c r="B3754" t="s">
+        <v>160</v>
+      </c>
+      <c r="C3754" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3754" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3754" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3754" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3754" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3755" x14ac:dyDescent="0.25">
+      <c r="A3755" t="s">
+        <v>161</v>
+      </c>
+      <c r="B3755" t="s">
+        <v>162</v>
+      </c>
+      <c r="C3755" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3755" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3755" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3755" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3755" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3756" x14ac:dyDescent="0.25">
+      <c r="A3756" t="s">
+        <v>163</v>
+      </c>
+      <c r="B3756" t="s">
+        <v>164</v>
+      </c>
+      <c r="C3756" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3756" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3756" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3756" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3756" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3757" x14ac:dyDescent="0.25">
+      <c r="A3757" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3757" t="s">
+        <v>166</v>
+      </c>
+      <c r="C3757" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3757" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3757" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3757" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3757" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3758" x14ac:dyDescent="0.25">
+      <c r="A3758" t="s">
+        <v>167</v>
+      </c>
+      <c r="B3758" t="s">
+        <v>168</v>
+      </c>
+      <c r="C3758" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3758" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3758" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3758" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3758" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3759" x14ac:dyDescent="0.25">
+      <c r="A3759" t="s">
+        <v>169</v>
+      </c>
+      <c r="B3759" t="s">
+        <v>170</v>
+      </c>
+      <c r="C3759" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3759" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3759" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3759" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3759" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3760" x14ac:dyDescent="0.25">
+      <c r="A3760" t="s">
+        <v>171</v>
+      </c>
+      <c r="B3760" t="s">
+        <v>172</v>
+      </c>
+      <c r="C3760" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3760" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3760" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3760" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3760" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3761" x14ac:dyDescent="0.25">
+      <c r="A3761" t="s">
+        <v>173</v>
+      </c>
+      <c r="B3761" t="s">
+        <v>174</v>
+      </c>
+      <c r="C3761" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3761" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3761" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3761" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3761" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3762" x14ac:dyDescent="0.25">
+      <c r="A3762" t="s">
+        <v>175</v>
+      </c>
+      <c r="B3762" t="s">
+        <v>176</v>
+      </c>
+      <c r="C3762" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3762" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3762" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3762" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3762" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3763" x14ac:dyDescent="0.25">
+      <c r="A3763" t="s">
+        <v>177</v>
+      </c>
+      <c r="B3763" t="s">
+        <v>178</v>
+      </c>
+      <c r="C3763" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3763" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3763" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3763" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3763" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3764" x14ac:dyDescent="0.25">
+      <c r="A3764" t="s">
+        <v>179</v>
+      </c>
+      <c r="B3764" t="s">
+        <v>180</v>
+      </c>
+      <c r="C3764" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3764" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3764" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3764" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3764" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3765" x14ac:dyDescent="0.25">
+      <c r="A3765" t="s">
+        <v>181</v>
+      </c>
+      <c r="B3765" t="s">
+        <v>182</v>
+      </c>
+      <c r="C3765" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3765" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3765" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3765" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3765" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3766" x14ac:dyDescent="0.25">
+      <c r="A3766" t="s">
+        <v>183</v>
+      </c>
+      <c r="B3766" t="s">
+        <v>184</v>
+      </c>
+      <c r="C3766" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3766" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3766" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3766" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3766" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3767" x14ac:dyDescent="0.25">
+      <c r="A3767" t="s">
+        <v>185</v>
+      </c>
+      <c r="B3767" t="s">
+        <v>186</v>
+      </c>
+      <c r="C3767" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3767" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3767" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3767" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3767" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3768" x14ac:dyDescent="0.25">
+      <c r="A3768" t="s">
+        <v>187</v>
+      </c>
+      <c r="B3768" t="s">
+        <v>188</v>
+      </c>
+      <c r="C3768" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3768" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3768" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3768" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3768" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3769" x14ac:dyDescent="0.25">
+      <c r="A3769" t="s">
+        <v>189</v>
+      </c>
+      <c r="B3769" t="s">
+        <v>190</v>
+      </c>
+      <c r="C3769" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3769" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3769" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3769" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3769" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3770" x14ac:dyDescent="0.25">
+      <c r="A3770" t="s">
+        <v>191</v>
+      </c>
+      <c r="B3770" t="s">
+        <v>192</v>
+      </c>
+      <c r="C3770" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3770" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3770" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3770" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3770" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3771" x14ac:dyDescent="0.25">
+      <c r="A3771" t="s">
+        <v>193</v>
+      </c>
+      <c r="B3771" t="s">
+        <v>194</v>
+      </c>
+      <c r="C3771" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3771" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3771" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3771" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3771" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3772" x14ac:dyDescent="0.25">
+      <c r="A3772" t="s">
+        <v>195</v>
+      </c>
+      <c r="B3772" t="s">
+        <v>196</v>
+      </c>
+      <c r="C3772" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3772" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3772" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3772" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3772" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3773" x14ac:dyDescent="0.25">
+      <c r="A3773" t="s">
+        <v>197</v>
+      </c>
+      <c r="B3773" t="s">
+        <v>198</v>
+      </c>
+      <c r="C3773" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3773" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3773" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3773" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3773" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3774" x14ac:dyDescent="0.25">
+      <c r="A3774" t="s">
+        <v>199</v>
+      </c>
+      <c r="B3774" t="s">
+        <v>200</v>
+      </c>
+      <c r="C3774" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3774" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3774" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3774" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3774" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3775" x14ac:dyDescent="0.25">
+      <c r="A3775" t="s">
+        <v>201</v>
+      </c>
+      <c r="B3775" t="s">
+        <v>202</v>
+      </c>
+      <c r="C3775" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3775" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3775" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3775" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3775" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3776" x14ac:dyDescent="0.25">
+      <c r="A3776" t="s">
+        <v>203</v>
+      </c>
+      <c r="B3776" t="s">
+        <v>204</v>
+      </c>
+      <c r="C3776" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3776" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3776" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3776" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3776" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3777" x14ac:dyDescent="0.25">
+      <c r="A3777" t="s">
+        <v>205</v>
+      </c>
+      <c r="B3777" t="s">
+        <v>206</v>
+      </c>
+      <c r="C3777" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3777" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3777" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3777" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3777" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3778" x14ac:dyDescent="0.25">
+      <c r="A3778" t="s">
+        <v>207</v>
+      </c>
+      <c r="B3778" t="s">
+        <v>208</v>
+      </c>
+      <c r="C3778" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3778" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3778" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3778" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3778" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3779" x14ac:dyDescent="0.25">
+      <c r="A3779" t="s">
+        <v>209</v>
+      </c>
+      <c r="B3779" t="s">
+        <v>210</v>
+      </c>
+      <c r="C3779" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3779" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3779" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3779" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3779" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3780" x14ac:dyDescent="0.25">
+      <c r="A3780" t="s">
+        <v>211</v>
+      </c>
+      <c r="B3780" t="s">
+        <v>212</v>
+      </c>
+      <c r="C3780" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3780" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3780" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3780" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3780" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3781" x14ac:dyDescent="0.25">
+      <c r="A3781" t="s">
+        <v>213</v>
+      </c>
+      <c r="B3781" t="s">
+        <v>214</v>
+      </c>
+      <c r="C3781" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3781" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3781" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3781" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3781" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3782" x14ac:dyDescent="0.25">
+      <c r="A3782" t="s">
+        <v>215</v>
+      </c>
+      <c r="B3782" t="s">
+        <v>216</v>
+      </c>
+      <c r="C3782" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3782" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3782" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3782" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3782" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3783" x14ac:dyDescent="0.25">
+      <c r="A3783" t="s">
+        <v>217</v>
+      </c>
+      <c r="B3783" t="s">
+        <v>218</v>
+      </c>
+      <c r="C3783" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3783" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3783" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3783" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3783" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3784" x14ac:dyDescent="0.25">
+      <c r="A3784" t="s">
+        <v>219</v>
+      </c>
+      <c r="B3784" t="s">
+        <v>220</v>
+      </c>
+      <c r="C3784" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3784" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3784" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3784" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3784" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3785" x14ac:dyDescent="0.25">
+      <c r="A3785" t="s">
+        <v>221</v>
+      </c>
+      <c r="B3785" t="s">
+        <v>222</v>
+      </c>
+      <c r="C3785" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3785" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3785" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3785" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3785" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3786" x14ac:dyDescent="0.25">
+      <c r="A3786" t="s">
+        <v>223</v>
+      </c>
+      <c r="B3786" t="s">
+        <v>224</v>
+      </c>
+      <c r="C3786" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3786" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3786" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3786" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3786" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3787" x14ac:dyDescent="0.25">
+      <c r="A3787" t="s">
+        <v>225</v>
+      </c>
+      <c r="B3787" t="s">
+        <v>226</v>
+      </c>
+      <c r="C3787" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3787" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3787" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3787" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3787" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3788" x14ac:dyDescent="0.25">
+      <c r="A3788" t="s">
+        <v>227</v>
+      </c>
+      <c r="B3788" t="s">
+        <v>228</v>
+      </c>
+      <c r="C3788" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3788" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3788" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3788" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3788" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3789" x14ac:dyDescent="0.25">
+      <c r="A3789" t="s">
+        <v>229</v>
+      </c>
+      <c r="B3789" t="s">
+        <v>230</v>
+      </c>
+      <c r="C3789" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3789" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3789" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3789" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3789" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3790" x14ac:dyDescent="0.25">
+      <c r="A3790" t="s">
+        <v>231</v>
+      </c>
+      <c r="B3790" t="s">
+        <v>232</v>
+      </c>
+      <c r="C3790" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3790" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3790" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3790" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3790" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3791" x14ac:dyDescent="0.25">
+      <c r="A3791" t="s">
+        <v>233</v>
+      </c>
+      <c r="B3791" t="s">
+        <v>234</v>
+      </c>
+      <c r="C3791" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3791" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3791" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3791" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3791" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3792" x14ac:dyDescent="0.25">
+      <c r="A3792" t="s">
+        <v>235</v>
+      </c>
+      <c r="B3792" t="s">
+        <v>236</v>
+      </c>
+      <c r="C3792" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3792" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3792" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3792" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3792" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3793" x14ac:dyDescent="0.25">
+      <c r="A3793" t="s">
+        <v>237</v>
+      </c>
+      <c r="B3793" t="s">
+        <v>238</v>
+      </c>
+      <c r="C3793" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3793" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3793" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3793" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3793" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3794" x14ac:dyDescent="0.25">
+      <c r="A3794" t="s">
+        <v>239</v>
+      </c>
+      <c r="B3794" t="s">
+        <v>240</v>
+      </c>
+      <c r="C3794" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3794" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3794" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3794" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3794" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3795" x14ac:dyDescent="0.25">
+      <c r="A3795" t="s">
+        <v>241</v>
+      </c>
+      <c r="B3795" t="s">
+        <v>242</v>
+      </c>
+      <c r="C3795" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3795" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3795" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3795" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3795" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3796" x14ac:dyDescent="0.25">
+      <c r="A3796" t="s">
+        <v>243</v>
+      </c>
+      <c r="B3796" t="s">
+        <v>244</v>
+      </c>
+      <c r="C3796" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3796" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3796" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3796" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3796" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3797" x14ac:dyDescent="0.25">
+      <c r="A3797" t="s">
+        <v>245</v>
+      </c>
+      <c r="B3797" t="s">
+        <v>246</v>
+      </c>
+      <c r="C3797" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3797" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3797" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3797" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3797" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3798" x14ac:dyDescent="0.25">
+      <c r="A3798" t="s">
+        <v>247</v>
+      </c>
+      <c r="B3798" t="s">
+        <v>248</v>
+      </c>
+      <c r="C3798" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3798" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3798" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3798" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3798" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3799" x14ac:dyDescent="0.25">
+      <c r="A3799" t="s">
+        <v>249</v>
+      </c>
+      <c r="B3799" t="s">
+        <v>250</v>
+      </c>
+      <c r="C3799" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3799" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3799" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3799" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3799" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3800" x14ac:dyDescent="0.25">
+      <c r="A3800" t="s">
+        <v>251</v>
+      </c>
+      <c r="B3800" t="s">
+        <v>252</v>
+      </c>
+      <c r="C3800" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3800" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3800" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3800" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3800" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3801" x14ac:dyDescent="0.25">
+      <c r="A3801" t="s">
+        <v>253</v>
+      </c>
+      <c r="B3801" t="s">
+        <v>254</v>
+      </c>
+      <c r="C3801" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3801" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3801" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3801" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3801" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3802" x14ac:dyDescent="0.25">
+      <c r="A3802" t="s">
+        <v>255</v>
+      </c>
+      <c r="B3802" t="s">
+        <v>256</v>
+      </c>
+      <c r="C3802" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3802" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3802" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3802" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3802" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3803" x14ac:dyDescent="0.25">
+      <c r="A3803" t="s">
+        <v>257</v>
+      </c>
+      <c r="B3803" t="s">
+        <v>258</v>
+      </c>
+      <c r="C3803" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3803" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3803" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3803" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3803" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3804" x14ac:dyDescent="0.25">
+      <c r="A3804" t="s">
+        <v>259</v>
+      </c>
+      <c r="B3804" t="s">
+        <v>260</v>
+      </c>
+      <c r="C3804" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3804" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3804" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3804" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3804" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3805" x14ac:dyDescent="0.25">
+      <c r="A3805" t="s">
+        <v>261</v>
+      </c>
+      <c r="B3805" t="s">
+        <v>262</v>
+      </c>
+      <c r="C3805" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3805" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3805" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3805" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3805" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3806" x14ac:dyDescent="0.25">
+      <c r="A3806" t="s">
+        <v>263</v>
+      </c>
+      <c r="B3806" t="s">
+        <v>264</v>
+      </c>
+      <c r="C3806" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3806" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3806" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3806" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3806" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3807" x14ac:dyDescent="0.25">
+      <c r="A3807" t="s">
+        <v>265</v>
+      </c>
+      <c r="B3807" t="s">
+        <v>266</v>
+      </c>
+      <c r="C3807" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3807" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3807" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3807" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3807" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3808" x14ac:dyDescent="0.25">
+      <c r="A3808" t="s">
+        <v>267</v>
+      </c>
+      <c r="B3808" t="s">
+        <v>268</v>
+      </c>
+      <c r="C3808" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3808" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3808" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3808" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3808" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3809" x14ac:dyDescent="0.25">
+      <c r="A3809" t="s">
+        <v>269</v>
+      </c>
+      <c r="B3809" t="s">
+        <v>270</v>
+      </c>
+      <c r="C3809" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3809" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3809" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3809" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3809" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3810" x14ac:dyDescent="0.25">
+      <c r="A3810" t="s">
+        <v>271</v>
+      </c>
+      <c r="B3810" t="s">
+        <v>272</v>
+      </c>
+      <c r="C3810" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3810" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3810" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3810" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3810" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3811" x14ac:dyDescent="0.25">
+      <c r="A3811" t="s">
+        <v>273</v>
+      </c>
+      <c r="B3811" t="s">
+        <v>274</v>
+      </c>
+      <c r="C3811" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3811" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3811" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3811" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3811" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3812" x14ac:dyDescent="0.25">
+      <c r="A3812" t="s">
+        <v>275</v>
+      </c>
+      <c r="B3812" t="s">
+        <v>276</v>
+      </c>
+      <c r="C3812" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3812" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3812" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3812" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3812" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3813" x14ac:dyDescent="0.25">
+      <c r="A3813" t="s">
+        <v>277</v>
+      </c>
+      <c r="B3813" t="s">
+        <v>278</v>
+      </c>
+      <c r="C3813" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3813" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3813" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3813" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3813" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="3814" x14ac:dyDescent="0.25">
+      <c r="A3814" t="s">
+        <v>279</v>
+      </c>
+      <c r="B3814" t="s">
+        <v>280</v>
+      </c>
+      <c r="C3814" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3814" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3814" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3814" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3814" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3815" x14ac:dyDescent="0.25">
+      <c r="A3815" t="s">
+        <v>281</v>
+      </c>
+      <c r="B3815" t="s">
+        <v>282</v>
+      </c>
+      <c r="C3815" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3815" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3815" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3815" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3815" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3816" x14ac:dyDescent="0.25">
+      <c r="A3816" t="s">
+        <v>283</v>
+      </c>
+      <c r="B3816" t="s">
+        <v>284</v>
+      </c>
+      <c r="C3816" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3816" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3816" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3816" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3816" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3817" x14ac:dyDescent="0.25">
+      <c r="A3817" t="s">
+        <v>285</v>
+      </c>
+      <c r="B3817" t="s">
+        <v>286</v>
+      </c>
+      <c r="C3817" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3817" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3817" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3817" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3817" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3818" x14ac:dyDescent="0.25">
+      <c r="A3818" t="s">
+        <v>287</v>
+      </c>
+      <c r="B3818" t="s">
+        <v>288</v>
+      </c>
+      <c r="C3818" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3818" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3818" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3818" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3818" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3819" x14ac:dyDescent="0.25">
+      <c r="A3819" t="s">
+        <v>289</v>
+      </c>
+      <c r="B3819" t="s">
+        <v>290</v>
+      </c>
+      <c r="C3819" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3819" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3819" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3819" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3819" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="3820" x14ac:dyDescent="0.25">
+      <c r="A3820" t="s">
+        <v>291</v>
+      </c>
+      <c r="B3820" t="s">
+        <v>292</v>
+      </c>
+      <c r="C3820" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3820" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3820" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3820" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3820" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3821" x14ac:dyDescent="0.25">
+      <c r="A3821" t="s">
+        <v>293</v>
+      </c>
+      <c r="B3821" t="s">
+        <v>294</v>
+      </c>
+      <c r="C3821" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3821" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3821" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3821" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3821" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3822" x14ac:dyDescent="0.25">
+      <c r="A3822" t="s">
+        <v>295</v>
+      </c>
+      <c r="B3822" t="s">
+        <v>296</v>
+      </c>
+      <c r="C3822" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3822" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3822" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3822" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3822" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3823" x14ac:dyDescent="0.25">
+      <c r="A3823" t="s">
+        <v>297</v>
+      </c>
+      <c r="B3823" t="s">
+        <v>298</v>
+      </c>
+      <c r="C3823" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3823" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3823" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3823" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3823" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3824" x14ac:dyDescent="0.25">
+      <c r="A3824" t="s">
+        <v>299</v>
+      </c>
+      <c r="B3824" t="s">
+        <v>300</v>
+      </c>
+      <c r="C3824" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3824" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3824" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3824" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3824" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="3825" x14ac:dyDescent="0.25">
+      <c r="A3825" t="s">
+        <v>301</v>
+      </c>
+      <c r="B3825" t="s">
+        <v>302</v>
+      </c>
+      <c r="C3825" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3825" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3825" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3825" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3825" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3826" x14ac:dyDescent="0.25">
+      <c r="A3826" t="s">
+        <v>303</v>
+      </c>
+      <c r="B3826" t="s">
+        <v>304</v>
+      </c>
+      <c r="C3826" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3826" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3826" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3826" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3826" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3827" x14ac:dyDescent="0.25">
+      <c r="A3827" t="s">
+        <v>305</v>
+      </c>
+      <c r="B3827" t="s">
+        <v>306</v>
+      </c>
+      <c r="C3827" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3827" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3827" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3827" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3827" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3828" x14ac:dyDescent="0.25">
+      <c r="A3828" t="s">
+        <v>307</v>
+      </c>
+      <c r="B3828" t="s">
+        <v>308</v>
+      </c>
+      <c r="C3828" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3828" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3828" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3828" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3828" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3829" x14ac:dyDescent="0.25">
+      <c r="A3829" t="s">
+        <v>309</v>
+      </c>
+      <c r="B3829" t="s">
+        <v>310</v>
+      </c>
+      <c r="C3829" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3829" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3829" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3829" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3829" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3830" x14ac:dyDescent="0.25">
+      <c r="A3830" t="s">
+        <v>311</v>
+      </c>
+      <c r="B3830" t="s">
+        <v>312</v>
+      </c>
+      <c r="C3830" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3830" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3830" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3830" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3830" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3831" x14ac:dyDescent="0.25">
+      <c r="A3831" t="s">
+        <v>313</v>
+      </c>
+      <c r="B3831" t="s">
+        <v>314</v>
+      </c>
+      <c r="C3831" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3831" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3831" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3831" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3831" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3832" x14ac:dyDescent="0.25">
+      <c r="A3832" t="s">
+        <v>315</v>
+      </c>
+      <c r="B3832" t="s">
+        <v>316</v>
+      </c>
+      <c r="C3832" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3832" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3832" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3832" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3832" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3833" x14ac:dyDescent="0.25">
+      <c r="A3833" t="s">
+        <v>317</v>
+      </c>
+      <c r="B3833" t="s">
+        <v>318</v>
+      </c>
+      <c r="C3833" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3833" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3833" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3833" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3833" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3834" x14ac:dyDescent="0.25">
+      <c r="A3834" t="s">
+        <v>319</v>
+      </c>
+      <c r="B3834" t="s">
+        <v>320</v>
+      </c>
+      <c r="C3834" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3834" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3834" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3834" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3834" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3835" x14ac:dyDescent="0.25">
+      <c r="A3835" t="s">
+        <v>321</v>
+      </c>
+      <c r="B3835" t="s">
+        <v>322</v>
+      </c>
+      <c r="C3835" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3835" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3835" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3835" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3835" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3836" x14ac:dyDescent="0.25">
+      <c r="A3836" t="s">
+        <v>323</v>
+      </c>
+      <c r="B3836" t="s">
+        <v>324</v>
+      </c>
+      <c r="C3836" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3836" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3836" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3836" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3836" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3837" x14ac:dyDescent="0.25">
+      <c r="A3837" t="s">
+        <v>325</v>
+      </c>
+      <c r="B3837" t="s">
+        <v>326</v>
+      </c>
+      <c r="C3837" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3837" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3837" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3837" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3837" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3838" x14ac:dyDescent="0.25">
+      <c r="A3838" t="s">
+        <v>327</v>
+      </c>
+      <c r="B3838" t="s">
+        <v>328</v>
+      </c>
+      <c r="C3838" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3838" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3838" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3838" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3838" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3839" x14ac:dyDescent="0.25">
+      <c r="A3839" t="s">
+        <v>329</v>
+      </c>
+      <c r="B3839" t="s">
+        <v>330</v>
+      </c>
+      <c r="C3839" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3839" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3839" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3839" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3839" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3840" x14ac:dyDescent="0.25">
+      <c r="A3840" t="s">
+        <v>331</v>
+      </c>
+      <c r="B3840" t="s">
+        <v>332</v>
+      </c>
+      <c r="C3840" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3840" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3840" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3840" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3840" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3841" x14ac:dyDescent="0.25">
+      <c r="A3841" t="s">
+        <v>333</v>
+      </c>
+      <c r="B3841" t="s">
+        <v>334</v>
+      </c>
+      <c r="C3841" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3841" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3841" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3841" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3841" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3842" x14ac:dyDescent="0.25">
+      <c r="A3842" t="s">
+        <v>335</v>
+      </c>
+      <c r="B3842" t="s">
+        <v>336</v>
+      </c>
+      <c r="C3842" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3842" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3842" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3842" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3842" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3843" x14ac:dyDescent="0.25">
+      <c r="A3843" t="s">
+        <v>337</v>
+      </c>
+      <c r="B3843" t="s">
+        <v>338</v>
+      </c>
+      <c r="C3843" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3843" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3843" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3843" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3843" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3844" x14ac:dyDescent="0.25">
+      <c r="A3844" t="s">
+        <v>339</v>
+      </c>
+      <c r="B3844" t="s">
+        <v>340</v>
+      </c>
+      <c r="C3844" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3844" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3844" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3844" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3844" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3845" x14ac:dyDescent="0.25">
+      <c r="A3845" t="s">
+        <v>404</v>
+      </c>
+      <c r="B3845" t="s">
+        <v>405</v>
+      </c>
+      <c r="C3845" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3845" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3845" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3845" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3845" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3846" x14ac:dyDescent="0.25">
+      <c r="A3846" t="s">
+        <v>341</v>
+      </c>
+      <c r="B3846" t="s">
+        <v>342</v>
+      </c>
+      <c r="C3846" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3846" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3846" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3846" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3846" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3847" x14ac:dyDescent="0.25">
+      <c r="A3847" t="s">
+        <v>343</v>
+      </c>
+      <c r="B3847" t="s">
+        <v>344</v>
+      </c>
+      <c r="C3847" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3847" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3847" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3847" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3847" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3848" x14ac:dyDescent="0.25">
+      <c r="A3848" t="s">
+        <v>345</v>
+      </c>
+      <c r="B3848" t="s">
+        <v>346</v>
+      </c>
+      <c r="C3848" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3848" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3848" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3848" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3848" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3849" x14ac:dyDescent="0.25">
+      <c r="A3849" t="s">
+        <v>347</v>
+      </c>
+      <c r="B3849" t="s">
+        <v>348</v>
+      </c>
+      <c r="C3849" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3849" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3849" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3849" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3849" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3850" x14ac:dyDescent="0.25">
+      <c r="A3850" t="s">
+        <v>349</v>
+      </c>
+      <c r="B3850" t="s">
+        <v>350</v>
+      </c>
+      <c r="C3850" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3850" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3850" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3850" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3850" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3851" x14ac:dyDescent="0.25">
+      <c r="A3851" t="s">
+        <v>351</v>
+      </c>
+      <c r="B3851" t="s">
+        <v>352</v>
+      </c>
+      <c r="C3851" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3851" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3851" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3851" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3851" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3852" x14ac:dyDescent="0.25">
+      <c r="A3852" t="s">
+        <v>353</v>
+      </c>
+      <c r="B3852" t="s">
+        <v>354</v>
+      </c>
+      <c r="C3852" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3852" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3852" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3852" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3852" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3853" x14ac:dyDescent="0.25">
+      <c r="A3853" t="s">
+        <v>355</v>
+      </c>
+      <c r="B3853" t="s">
+        <v>356</v>
+      </c>
+      <c r="C3853" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3853" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3853" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3853" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3853" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3854" x14ac:dyDescent="0.25">
+      <c r="A3854" t="s">
+        <v>357</v>
+      </c>
+      <c r="B3854" t="s">
+        <v>358</v>
+      </c>
+      <c r="C3854" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3854" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3854" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3854" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3854" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3855" x14ac:dyDescent="0.25">
+      <c r="A3855" t="s">
+        <v>359</v>
+      </c>
+      <c r="B3855" t="s">
+        <v>360</v>
+      </c>
+      <c r="C3855" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3855" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3855" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3855" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3855" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3856" x14ac:dyDescent="0.25">
+      <c r="A3856" t="s">
+        <v>361</v>
+      </c>
+      <c r="B3856" t="s">
+        <v>362</v>
+      </c>
+      <c r="C3856" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3856" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3856" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3856" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3856" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3857" x14ac:dyDescent="0.25">
+      <c r="A3857" t="s">
+        <v>363</v>
+      </c>
+      <c r="B3857" t="s">
+        <v>364</v>
+      </c>
+      <c r="C3857" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3857" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3857" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3857" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3857" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3858" x14ac:dyDescent="0.25">
+      <c r="A3858" t="s">
+        <v>365</v>
+      </c>
+      <c r="B3858" t="s">
+        <v>366</v>
+      </c>
+      <c r="C3858" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3858" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3858" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3858" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3858" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3859" x14ac:dyDescent="0.25">
+      <c r="A3859" t="s">
+        <v>367</v>
+      </c>
+      <c r="B3859" t="s">
+        <v>368</v>
+      </c>
+      <c r="C3859" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3859" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3859" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3859" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3859" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3860" x14ac:dyDescent="0.25">
+      <c r="A3860" t="s">
+        <v>369</v>
+      </c>
+      <c r="B3860" t="s">
+        <v>370</v>
+      </c>
+      <c r="C3860" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3860" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3860" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3860" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3860" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3861" x14ac:dyDescent="0.25">
+      <c r="A3861" t="s">
+        <v>371</v>
+      </c>
+      <c r="B3861" t="s">
+        <v>372</v>
+      </c>
+      <c r="C3861" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3861" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3861" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3861" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3861" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3862" x14ac:dyDescent="0.25">
+      <c r="A3862" t="s">
+        <v>373</v>
+      </c>
+      <c r="B3862" t="s">
+        <v>374</v>
+      </c>
+      <c r="C3862" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3862" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3862" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3862" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3862" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3863" x14ac:dyDescent="0.25">
+      <c r="A3863" t="s">
+        <v>375</v>
+      </c>
+      <c r="B3863" t="s">
+        <v>376</v>
+      </c>
+      <c r="C3863" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3863" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3863" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3863" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3863" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3864" x14ac:dyDescent="0.25">
+      <c r="A3864" t="s">
+        <v>377</v>
+      </c>
+      <c r="B3864" t="s">
+        <v>378</v>
+      </c>
+      <c r="C3864" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3864" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3864" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3864" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3864" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3865" x14ac:dyDescent="0.25">
+      <c r="A3865" t="s">
+        <v>379</v>
+      </c>
+      <c r="B3865" t="s">
+        <v>380</v>
+      </c>
+      <c r="C3865" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3865" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3865" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3865" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3865" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3866" x14ac:dyDescent="0.25">
+      <c r="A3866" t="s">
+        <v>381</v>
+      </c>
+      <c r="B3866" t="s">
+        <v>382</v>
+      </c>
+      <c r="C3866" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3866" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3866" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3866" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3866" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3867" x14ac:dyDescent="0.25">
+      <c r="A3867" t="s">
+        <v>383</v>
+      </c>
+      <c r="B3867" t="s">
+        <v>384</v>
+      </c>
+      <c r="C3867" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3867" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3867" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3867" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3867" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3868" x14ac:dyDescent="0.25">
+      <c r="A3868" t="s">
+        <v>385</v>
+      </c>
+      <c r="B3868" t="s">
+        <v>386</v>
+      </c>
+      <c r="C3868" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3868" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3868" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3868" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3868" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3869" x14ac:dyDescent="0.25">
+      <c r="A3869" t="s">
+        <v>387</v>
+      </c>
+      <c r="B3869" t="s">
+        <v>388</v>
+      </c>
+      <c r="C3869" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3869" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3869" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3869" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3869" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3870" x14ac:dyDescent="0.25">
+      <c r="A3870" t="s">
+        <v>389</v>
+      </c>
+      <c r="B3870" t="s">
+        <v>390</v>
+      </c>
+      <c r="C3870" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3870" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3870" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3870" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3870" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3871" x14ac:dyDescent="0.25">
+      <c r="A3871" t="s">
+        <v>391</v>
+      </c>
+      <c r="B3871" t="s">
+        <v>392</v>
+      </c>
+      <c r="C3871" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3871" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3871" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3871" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3871" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3872" x14ac:dyDescent="0.25">
+      <c r="A3872" t="s">
+        <v>393</v>
+      </c>
+      <c r="B3872" t="s">
+        <v>394</v>
+      </c>
+      <c r="C3872" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3872" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3872" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3872" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3872" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3873" x14ac:dyDescent="0.25">
+      <c r="A3873" t="s">
+        <v>395</v>
+      </c>
+      <c r="B3873" t="s">
+        <v>396</v>
+      </c>
+      <c r="C3873" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3873" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3873" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3873" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3873" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3874" x14ac:dyDescent="0.25">
+      <c r="A3874" t="s">
+        <v>397</v>
+      </c>
+      <c r="B3874" t="s">
+        <v>398</v>
+      </c>
+      <c r="C3874" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3874" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3874" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3874" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3874" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3875" x14ac:dyDescent="0.25">
+      <c r="A3875" t="s">
+        <v>399</v>
+      </c>
+      <c r="B3875" t="s">
+        <v>400</v>
+      </c>
+      <c r="C3875" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3875" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3875" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3875" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3875" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3876" x14ac:dyDescent="0.25">
+      <c r="A3876" t="s">
+        <v>401</v>
+      </c>
+      <c r="B3876" t="s">
+        <v>402</v>
+      </c>
+      <c r="C3876" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3876" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E3876" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3876" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3876" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3877" x14ac:dyDescent="0.25">
+      <c r="A3877" t="s">
         <v>407</v>
       </c>
     </row>
@@ -86176,10 +90652,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr x14ac:dyDescent="0.25" customHeight="1" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="22.714285714285715" bestFit="1"/>
+    <col min="1" max="1" customWidth="1" width="40.714285714285715" bestFit="1"/>
   </cols>
   <sheetData>
     <row r="1" x14ac:dyDescent="0.25">
@@ -86252,6 +90728,14 @@
       </c>
       <c r="B9" s="2" t="s">
         <v>437</v>
+      </c>
+    </row>
+    <row r="10" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>439</v>
       </c>
     </row>
   </sheetData>
@@ -86261,7 +90745,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr x14ac:dyDescent="0.25" customHeight="1" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="155.71428571428572" bestFit="1"/>
@@ -86269,7 +90753,12 @@
   <sheetData>
     <row r="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>438</v>
+        <v>440</v>
+      </c>
+    </row>
+    <row r="2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>441</v>
       </c>
     </row>
   </sheetData>

</xml_diff>